<commit_message>
fixed excel input files with new circles validation and formatting
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template (with sample inputs).xlsx
+++ b/docs/inputs/input_template (with sample inputs).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BC16DC-CF57-2044-B849-9FF18EE44AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83688958-FECD-084D-B75C-89BB7F00E5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24520" yWindow="2880" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="24520" yWindow="2880" windowWidth="34200" windowHeight="20240" activeTab="5" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1084,7 +1084,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -10436,32 +10457,32 @@
     <mergeCell ref="R7:V7"/>
   </mergeCells>
   <conditionalFormatting sqref="E9:F50">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="6" priority="4">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:N50">
-    <cfRule type="expression" dxfId="2" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="4" priority="13">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="3" priority="8">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12138,12 +12159,24 @@
       <c r="N16" s="1"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D12" xr:uid="{06E9E004-FC39-FE49-926A-912F810F5089}">
+  <conditionalFormatting sqref="E3:E42">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>OR($D3="Intercept", $D3="Radius")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:G42">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>OR($D3="Depth",$D3="Radius")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H42">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>OR($D3="Depth",$D3="Intercept")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D52" xr:uid="{7F956FD6-0589-5E4E-B392-27403BB6B3EC}">
       <formula1>$J$3:$J$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D4" xr:uid="{AEFC92A9-AB07-FF4B-9461-938B9BDCD07D}">
-      <formula1>$J$5:$J$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
new version of template. fixed conditional formatting error
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template (with sample inputs).xlsx
+++ b/docs/inputs/input_template (with sample inputs).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83688958-FECD-084D-B75C-89BB7F00E5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E5A92E-9DBF-4A42-A886-0C898438F60D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24520" yWindow="2880" windowWidth="34200" windowHeight="20240" activeTab="5" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="7820" yWindow="3500" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1053,13 +1053,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1084,25 +1084,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="15">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
+          <bgColor theme="2" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1145,6 +1145,48 @@
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8144,7 +8186,7 @@
         <v>78</v>
       </c>
       <c r="D5" s="35">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -9741,16 +9783,18 @@
         <v>120</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E10" s="3">
+        <v>200</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3">
         <v>100</v>
       </c>
-      <c r="F10" s="3">
-        <v>32</v>
-      </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="3">
+        <v>50</v>
+      </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3" t="s">
@@ -10456,33 +10500,33 @@
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="R7:V7"/>
   </mergeCells>
-  <conditionalFormatting sqref="E9:F50">
-    <cfRule type="expression" dxfId="8" priority="3">
+  <conditionalFormatting sqref="F9:F50">
+    <cfRule type="expression" dxfId="11" priority="3" stopIfTrue="1">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="6" priority="4">
+    <cfRule type="expression" dxfId="9" priority="4">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M9:N50">
-    <cfRule type="expression" dxfId="5" priority="6">
+  <conditionalFormatting sqref="N9:N50">
+    <cfRule type="expression" dxfId="8" priority="6" stopIfTrue="1">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="4" priority="13">
+    <cfRule type="expression" dxfId="7" priority="13">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="3" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10536,74 +10580,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="D4" s="45" t="s">
+      <c r="B4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="G4" s="45" t="s">
+      <c r="E4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="45"/>
-      <c r="J4" s="45" t="s">
+      <c r="H4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="M4" s="45" t="s">
+      <c r="K4" s="47"/>
+      <c r="M4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="45"/>
-      <c r="P4" s="45" t="s">
+      <c r="N4" s="47"/>
+      <c r="P4" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="45"/>
+      <c r="Q4" s="47"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="45"/>
+      <c r="T4" s="47"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="45"/>
+      <c r="W4" s="47"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="45" t="s">
+      <c r="Y4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="45"/>
+      <c r="Z4" s="47"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="45" t="s">
+      <c r="AB4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="45"/>
-      <c r="AE4" s="45" t="s">
+      <c r="AC4" s="47"/>
+      <c r="AE4" s="47" t="s">
         <v>115</v>
       </c>
-      <c r="AF4" s="45"/>
+      <c r="AF4" s="47"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="45" t="s">
+      <c r="AH4" s="47" t="s">
         <v>116</v>
       </c>
-      <c r="AI4" s="45"/>
+      <c r="AI4" s="47"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="45" t="s">
+      <c r="AK4" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="AL4" s="45"/>
+      <c r="AL4" s="47"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="45" t="s">
+      <c r="AN4" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="AO4" s="45"/>
+      <c r="AO4" s="47"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="45" t="s">
+      <c r="AQ4" s="47" t="s">
         <v>119</v>
       </c>
-      <c r="AR4" s="45"/>
+      <c r="AR4" s="47"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -10706,89 +10750,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="45" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Silt</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="46"/>
+      <c r="D6" s="45" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Sand</v>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="46"/>
+      <c r="G6" s="45" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Clay</v>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="46"/>
+      <c r="J6" s="45" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="46"/>
+      <c r="M6" s="45" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="46"/>
+      <c r="P6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="46"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="45" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="46"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="45" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="46"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="46"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="46"/>
+      <c r="AE6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="46"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="46"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="46"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="46"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="46"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11724,36 +11768,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12160,17 +12204,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="14" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="13" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>